<commit_message>
Rewrite Sugar News 2026-08-30 summary
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-30.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-30.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="162.6" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,46 +513,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度政府公布食糖价格和市场流通，糖价或相关政策基准为Rs 60。印度食糖价格上涨说明现货供应偏紧或节前需求增强，价格下跌则说明供应压力或需求转弱正在传导到现货端。来源：The New Indian Express（https://www.newindianexpress.com/india/2026/Aug/30/sugar-prices-stay-above-rs-60kg-in-most-markets-despite-centres-measures-to-curb-rise）。影响：利多糖价</t>
+          <t>印度消费者事务部数据显示，8月30日全印食糖平均零售价为₹64.24/kg，较一周前₹63.12/kg上涨1.77%，较一个月前上涨30%，同比上涨38.63%；批发均价为₹59.73/kg，较一周前₹58.66/kg继续上涨。零售和批发价格在政府允许100万吨原糖免税进口、收紧批量用户和经销商库存限制、此前禁止出口后仍维持高位，说明节前需求和产量下修造成印度国内现货偏紧，对印度国内糖价利多。印度2025/26榨季食糖产量预估为3060万吨、低于此前3430万吨，年消费约2800-2850万吨，低产预期会压缩出口余量并支撑国际糖价。来源：The New Indian Express（https://www.newindianexpress.com/india/2026/Aug/30/sugar-prices-stay-above-rs-60kg-in-most-markets-despite-centres-measures-to-curb-rise）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利多：现货或出厂报价上涨反映阶段性供应偏紧或采购需求增强，会支撑短期糖价。</t>
+          <t>利多：印度零售和批发糖价在进口、库存限制和出口禁令后仍上涨，说明国内可用糖源偏紧，产量预估下修进一步压缩出口余量并支撑糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="180" customHeight="1" s="2">
+    <row r="3" ht="116.4" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度政府公布食糖价格和市场流通，糖价或相关政策基准为₹60、E10。印度食糖价格上涨说明现货供应偏紧或节前需求增强，价格下跌则说明供应压力或需求转弱正在传导到现货端。来源：Livemint（https://www.livemint.com/money/personal-finance/sugar-prices-remain-above-rs-60-per-kg-in-india-despite-govt-measures-festive-season-city-wise-cost-mumbai-delhi-chennai-11788106922471.html）。影响：中性</t>
+          <t>泰国气象局8月30日预报，乌隆他尼、加拉信、黎府、甘烹碧、素可泰、彭世洛、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。泰国甘蔗仍处生长期，雷阵雨和局地大雨有利于补充土壤水分、改善墒情，促进单产形成并提高后期甘蔗及食糖供应预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>中性：价格信息缺少明确涨跌幅或区域基准，暂不改变供需判断。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="125.2" customHeight="1" s="2">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>泰国气象局预报（2026-08-30），乌隆他尼、加拉信、黎府、甘烹碧、素可泰、彭世洛、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+          <t>利空：泰国甘蔗生长期降雨有利于补充土壤水分、改善墒情并促进单产形成，从而增加未来甘蔗及食糖供应预期。</t>
         </is>
       </c>
     </row>

</xml_diff>